<commit_message>
Intial commit for finance dashboard project version 3
</commit_message>
<xml_diff>
--- a/finance-dashboard/excel_upload_template.xlsx
+++ b/finance-dashboard/excel_upload_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROJECT\FINANCE\finance-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9604C572-AD66-4F82-A4BB-0C04F8508BD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37095A6F-9380-4B73-BDCA-DC2DAC341344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="696" yWindow="696" windowWidth="15360" windowHeight="8040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="income" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="19">
   <si>
     <t>source</t>
   </si>
@@ -82,21 +82,15 @@
   </si>
   <si>
     <t>rental_income</t>
-  </si>
-  <si>
-    <t>INR</t>
-  </si>
-  <si>
-    <t>personal</t>
-  </si>
-  <si>
-    <t>2026-04-18</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -109,6 +103,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,11 +141,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -483,8 +479,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
@@ -502,6 +501,39 @@
       <c r="E1" s="1" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D4" s="2"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D7" s="2"/>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D16" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -606,7 +638,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
@@ -627,20 +659,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>400</v>
-      </c>
-      <c r="B2" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" t="s">
-        <v>20</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>